<commit_message>
Add 2026-09-27 part-time job watch digest
8 new within-15-mile listings, including the first Southampton-specific
Asda leads. KFC excluded per Adam's preference.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014mqK3D6nA4AdBsbRvpiLt1
</commit_message>
<xml_diff>
--- a/parttime-job-watch/Southampton_PartTime_Jobs_Tracker.xlsx
+++ b/parttime-job-watch/Southampton_PartTime_Jobs_Tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -560,7 +560,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -623,7 +622,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -686,7 +684,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -749,7 +746,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -812,7 +808,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -875,7 +870,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -938,7 +932,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1001,7 +994,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1064,7 +1056,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1127,7 +1118,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1190,7 +1180,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1253,7 +1242,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1316,7 +1304,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1379,7 +1366,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1442,7 +1428,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1505,7 +1490,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1568,7 +1552,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1631,7 +1614,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1694,7 +1676,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1757,7 +1738,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1820,7 +1800,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1883,7 +1862,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1946,7 +1924,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2009,7 +1986,6 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2072,7 +2048,510 @@
           <t>2026-09-13</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>NViro</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Weekend Cleaner</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aar7k7mmvsgt</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Atlas Hotels Group Ltd</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Team Member Cook</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aatgtljb4khr</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Wacky Kingdom</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Weekend Cleaner (part-time)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aadbshq4lzgk</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Pro-Football Academy Ltd</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Football Coach</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aadkfcr9f2zd</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Costa (Scoffs Group)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Costa Barista</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aayw6vzxqdtl</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Asda</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Service Colleague (Express)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Not stated (listed Permanent)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aax47rjxyfgg</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Asda</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Service Colleague (Food Services)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Not stated (listed Permanent)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aadnyd8ffjhv</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Colleague - Southampton Superstore</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Nursling</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>~4</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aajzgy7dm8cv</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2085,7 +2564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2112,6 +2591,18 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Full daily Indeed-only sweep (KFC excluded). 8 new within-15-mile listings, including the first two Southampton-specific Asda leads (Express, Food Services). Matalan, Sainsbury's, McDonald's, Showcase Cinemas, Vue Cinemas, Hollywood Bowl, IKEA, Lidl remain confirmed gaps or thin on Indeed today.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 2026-10-11 part-time job watch digest
10 new within-15-mile listings, including the start of Tesco's Christmas
"Festive Colleague" seasonal hiring wave across several nearby branches.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014mqK3D6nA4AdBsbRvpiLt1
</commit_message>
<xml_diff>
--- a/parttime-job-watch/Southampton_PartTime_Jobs_Tracker.xlsx
+++ b/parttime-job-watch/Southampton_PartTime_Jobs_Tracker.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2110,7 +2110,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2173,7 +2172,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2236,7 +2234,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2299,7 +2296,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2362,7 +2358,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2425,7 +2420,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2488,7 +2482,6 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2551,7 +2544,636 @@
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>West End Parish Council</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Cafe Assistant</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>~5</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Not stated (listed Permanent)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aamzyjp2b6bc</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Popsi's</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Pizza Chef</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Not stated (listed Permanent)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa6xzrb8ytfl</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Matalan</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>General Sales Assistant (Perm)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Eastleigh</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>~7</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aabpz76mfb42</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Costa (inMotion)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Barista Costa Coffee</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>~2</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aayclf9rqfdk</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Festive Colleague - Days - Hythe</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hythe</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aagywkzgjct9</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Festive Colleague - Twilights - Whiteley Superstore</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Whiteley</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>~9</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aal68qy7hyhq</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Festive Colleague - Nights - Bursledon Towers Extra</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Bursledon</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>~6</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aaqshrfjhnxb</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Colleague - Winchester Extra</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Winchester</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>~12</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa8r44jlvqpj</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Tesco</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Festive Colleague - Express</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Fordingbridge</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>~13</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aahy48jrnbcl</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Asda</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Service Colleague (Express)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Eastleigh</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>~7</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Not stated (listed Permanent)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>not stated</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://to.indeed.com/aa6dv9wbtjmd</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2564,7 +3186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2603,6 +3225,18 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Full daily Indeed-only sweep (KFC excluded). 10 new within-15-mile listings. Notable: Tesco has kicked off a Christmas 'Festive Colleague' seasonal hiring wave across several nearby branches (Hythe, Whiteley, Bursledon, Winchester, Fordingbridge) - worth flagging to Adam as a seasonal opportunity window. Boots, Sainsbury's, McDonald's, Showcase Cinemas, Vue Cinemas, Hollywood Bowl (only Portsmouth, out of range), IKEA remain confirmed gaps or out of range on Indeed today.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>